<commit_message>
Combined scan results 2026-08-28
</commit_message>
<xml_diff>
--- a/results/2026-08-28.xlsx
+++ b/results/2026-08-28.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,7 +453,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ABSI</t>
+          <t>AFRM</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -472,13 +472,13 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>AGYS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ABUS</t>
+          <t>ABSI</t>
         </is>
       </c>
     </row>
@@ -486,18 +486,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IMTX</t>
+          <t>CTMX</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AQST</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ACHV</t>
+          <t>ABUS</t>
         </is>
       </c>
     </row>
@@ -505,12 +505,12 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>INTR</t>
+          <t>IMTX</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AXGN</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -529,13 +529,13 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AYA</t>
+          <t>AXGN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ARGX</t>
+          <t>AQST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CACC</t>
+          <t>AYA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>ARGX</t>
         </is>
       </c>
     </row>
@@ -559,13 +559,13 @@
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CADL</t>
+          <t>BCRX</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>AU</t>
         </is>
       </c>
     </row>
@@ -574,13 +574,13 @@
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>BGC</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BGC</t>
+          <t>AVAH</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CLPT</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -610,7 +610,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CMPS</t>
+          <t>CACC</t>
         </is>
       </c>
     </row>
@@ -619,13 +619,13 @@
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CRON</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>CADL</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>CGAU</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>CLPT</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FCFS</t>
+          <t>CMPS</t>
         </is>
       </c>
     </row>
@@ -679,13 +679,13 @@
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FRHC</t>
+          <t>CRDO</t>
         </is>
       </c>
     </row>
@@ -694,13 +694,13 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>EZPW</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -709,13 +709,13 @@
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GEN</t>
+          <t>FRHC</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>CSX</t>
         </is>
       </c>
     </row>
@@ -724,13 +724,13 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HSIC</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
@@ -739,13 +739,13 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>IMMX</t>
+          <t>FCFS</t>
         </is>
       </c>
     </row>
@@ -754,13 +754,13 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>GEN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>IRON</t>
+          <t>GH</t>
         </is>
       </c>
     </row>
@@ -769,13 +769,13 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>IBKR</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>GILD</t>
         </is>
       </c>
     </row>
@@ -784,13 +784,13 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>IBKR</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MELI</t>
+          <t>GMAB</t>
         </is>
       </c>
     </row>
@@ -799,13 +799,13 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>IDYA</t>
+          <t>IBRX</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>NDSN</t>
+          <t>HOOD</t>
         </is>
       </c>
     </row>
@@ -814,13 +814,13 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>IFRX</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>NEXT</t>
+          <t>HSIC</t>
         </is>
       </c>
     </row>
@@ -829,13 +829,13 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>INBX</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>IDYA</t>
         </is>
       </c>
     </row>
@@ -844,13 +844,13 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>INBX</t>
+          <t>IRON</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>IFRX</t>
         </is>
       </c>
     </row>
@@ -859,13 +859,13 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>KRYS</t>
+          <t>KRNY</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>IMMX</t>
         </is>
       </c>
     </row>
@@ -874,13 +874,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>KRYS</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>JOYY</t>
         </is>
       </c>
     </row>
@@ -889,13 +889,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MDGL</t>
+          <t>LECO</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>LPTH</t>
         </is>
       </c>
     </row>
@@ -904,13 +904,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>PSNL</t>
+          <t>LTRX</t>
         </is>
       </c>
     </row>
@@ -919,13 +919,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>MDGL</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PVLA</t>
+          <t>MRVL</t>
         </is>
       </c>
     </row>
@@ -934,13 +934,13 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>NEO</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>QURE</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
@@ -949,13 +949,13 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>NEO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>REAX</t>
+          <t>NTRA</t>
         </is>
       </c>
     </row>
@@ -964,13 +964,13 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>NEXT</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>RGLD</t>
+          <t>NVDA</t>
         </is>
       </c>
     </row>
@@ -979,13 +979,13 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>NWS</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>OVID</t>
         </is>
       </c>
     </row>
@@ -994,13 +994,13 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SBRA</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>PANW</t>
         </is>
       </c>
     </row>
@@ -1009,13 +1009,13 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>OKTA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>RZLT</t>
+          <t>PHVS</t>
         </is>
       </c>
     </row>
@@ -1024,13 +1024,13 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SHC</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>PLTR</t>
         </is>
       </c>
     </row>
@@ -1039,13 +1039,13 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SLS</t>
+          <t>PTEN</t>
         </is>
       </c>
     </row>
@@ -1054,13 +1054,13 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SLDB</t>
+          <t>ROIV</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SRRK</t>
+          <t>REAX</t>
         </is>
       </c>
     </row>
@@ -1069,13 +1069,13 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SMTC</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SSRM</t>
+          <t>RGLD</t>
         </is>
       </c>
     </row>
@@ -1084,46 +1084,151 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>RPRX</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SLAB</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>TGTX</t>
+          <t>RZLT</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>SLDB</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>SBLK</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
+          <t>SBRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SMTC</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SEIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>TGTX</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SRRK</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SSRM</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>TRMD</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
           <t>TRLV</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>XNCR</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1166,182 +1271,584 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SKHY</t>
+          <t>BTBT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ASST</t>
+          <t>AVTR</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SPCX</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BULL</t>
+          <t>AVAH</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>SKHY</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>ADPT</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>IONS</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CELH</t>
+          <t>SPCX</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>BTU</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>BSY</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CHYM</t>
+          <t>BRZE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>DBX</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>BULL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>COIN</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>DOCU</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GEN</t>
+          <t>ASST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GTLB</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+          <t>CHYM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FIVE</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GLXY</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>GEN</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>INFQ</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>DXCM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>FROG</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PTEN</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MSTR</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>EXE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GENB</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SLS</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EXLS</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>BLSH</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FRSH</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MNDY</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>KMB</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>GILD</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CCEP</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MRSH</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>HTFL</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MTCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LFST</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>NAVN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CG</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NCNO</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>NESR</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>NWSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CHTR</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PGY</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PEGA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>COIN</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PTEN</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TMC</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>STRC</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PURR</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>EXEL</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>LITE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>FIVN</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RVMD</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SSRM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PAYX</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>PSKY</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>FWONK</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
           <t>SOFI</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>HALO</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SRPT</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>KURA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ROIV</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ALM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SBET</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>TRI</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TECH</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CRML</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TPG</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PAGP</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>RUM</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>